<commit_message>
Just change the datatype inferance by pl, causing some erros in the modelo column of the griglia file
</commit_message>
<xml_diff>
--- a/Map Opeperation/tb_de_para.xlsx
+++ b/Map Opeperation/tb_de_para.xlsx
@@ -3075,7 +3075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3103,148 +3103,126 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ELT(BSG12)</t>
+          <t>KW(125)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TIPO ELETTRIFICAZIONE</t>
+          <t>Potenza max KW</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Maximum power kW</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MHEV</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>KW(125)</t>
+          <t>L(L11)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Potenza max KW</t>
+          <t>Livello Allestimento</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Maximum power kW</t>
+          <t>Trim Level</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>LL5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>L(L11)</t>
+          <t>M(00)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Livello Allestimento</t>
+          <t>Marchio</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Trim Level</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>LL5</t>
-        </is>
-      </c>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>M(00)</t>
+          <t>T(ASP)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Marchio</t>
+          <t>Caratteristiche Motore</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Engine Features</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sovralimentato Turbo</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T(ASP)</t>
+          <t>TC(PKDC)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Caratteristiche Motore</t>
+          <t>Numero Porte</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Engine Features</t>
+          <t>Number of doors</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sovralimentato Turbo</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TC(PKDC)</t>
+          <t>TT(4X2)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Numero Porte</t>
+          <t>Tipo Trazione</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Number of doors</t>
+          <t>Traction type</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TT(4X2)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Tipo Trazione</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Traction type</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
         <is>
           <t>FWD</t>
         </is>

</xml_diff>